<commit_message>
update asturias mancha quesera
</commit_message>
<xml_diff>
--- a/posts/2026-04-26_asturias-mancha-quesera/AOC-Mancha_quesera_europa_update-claude-202604.xlsx
+++ b/posts/2026-04-26_asturias-mancha-quesera/AOC-Mancha_quesera_europa_update-claude-202604.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/blog-trabajo/asturias-mancha-quesera/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanr\GitHub\blog\posts\2026-04-26_asturias-mancha-quesera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{A835B32E-AF8A-43C3-A7DE-085E6D9B2406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{603DDBE3-EF76-45CF-85D3-22C2BA41E371}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1FD8A8-9953-4FFB-BAAD-C0E12AA059BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5190" yWindow="3135" windowWidth="17820" windowHeight="11190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Prod por pais" sheetId="1" r:id="rId1"/>
@@ -2697,7 +2697,7 @@
       <name val="Inherit"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2794,8 +2794,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F8F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -2980,11 +2986,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDFE2E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDFE2E5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDFE2E5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDFE2E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3222,19 +3243,25 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="17" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3431,10 +3458,6 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3685,7 +3708,7 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="13.140625" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
@@ -3695,7 +3718,7 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="12.75">
+    <row r="1" spans="1:8" ht="13.5" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3721,12 +3744,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="12.75">
+    <row r="2" spans="1:8" ht="13.5" thickBot="1">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="3">
-        <v>59000000</v>
+      <c r="B2" s="101">
+        <v>58957347</v>
       </c>
       <c r="C2" s="4">
         <v>301340</v>
@@ -3738,7 +3761,7 @@
         <v>620000</v>
       </c>
       <c r="F2" s="2">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G2" s="3">
         <v>1800</v>
@@ -3747,12 +3770,12 @@
         <v>800</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="12.75">
+    <row r="3" spans="1:8" ht="13.5" thickBot="1">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3">
-        <v>17877000</v>
+      <c r="B3" s="102">
+        <v>17993485</v>
       </c>
       <c r="C3" s="4">
         <v>41543</v>
@@ -3764,7 +3787,7 @@
         <v>303000</v>
       </c>
       <c r="F3" s="2">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G3" s="3">
         <v>300</v>
@@ -3773,12 +3796,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="12.75">
+    <row r="4" spans="1:8" ht="13.5" thickBot="1">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3">
-        <v>68000000</v>
+      <c r="B4" s="102">
+        <v>68775952</v>
       </c>
       <c r="C4" s="4">
         <v>551695</v>
@@ -3801,12 +3824,12 @@
         <v>484</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="12.75">
+    <row r="5" spans="1:8" ht="13.5" thickBot="1">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3">
-        <v>84524000</v>
+      <c r="B5" s="102">
+        <v>83516593</v>
       </c>
       <c r="C5" s="4">
         <v>357580</v>
@@ -3827,12 +3850,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="12.75">
+    <row r="6" spans="1:8" ht="13.5" thickBot="1">
       <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="3">
-        <v>10300000</v>
+      <c r="B6" s="101">
+        <v>10374050</v>
       </c>
       <c r="C6" s="3">
         <v>131957</v>
@@ -3853,12 +3876,12 @@
         <v>370</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="12.75">
+    <row r="7" spans="1:8" ht="13.5" thickBot="1">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3">
-        <v>8900000</v>
+      <c r="B7" s="101">
+        <v>9006644</v>
       </c>
       <c r="C7" s="4">
         <v>41285</v>
@@ -3879,12 +3902,12 @@
         <v>500</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="12.75">
+    <row r="8" spans="1:8" ht="13.5" thickBot="1">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3">
-        <v>47700000</v>
+      <c r="B8" s="101">
+        <v>48873996</v>
       </c>
       <c r="C8" s="3">
         <v>505990</v>
@@ -3905,12 +3928,12 @@
         <v>464</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="12.75">
+    <row r="9" spans="1:8" ht="13.5" thickBot="1">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3">
-        <v>9100000</v>
+      <c r="B9" s="101">
+        <v>9177982</v>
       </c>
       <c r="C9" s="3">
         <v>83871</v>
@@ -3931,12 +3954,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="12.75">
+    <row r="10" spans="1:8" ht="13.5" thickBot="1">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="3">
-        <v>5944000</v>
+      <c r="B10" s="101">
+        <v>5976992</v>
       </c>
       <c r="C10" s="4">
         <v>42933</v>
@@ -3957,23 +3980,23 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="12.75">
+    <row r="11" spans="1:8" ht="13.5" thickBot="1">
       <c r="A11" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="B11" s="3">
-        <v>1200000</v>
+        <v>19</v>
+      </c>
+      <c r="B11" s="102">
+        <v>5395980</v>
       </c>
       <c r="C11" s="3">
-        <v>9251</v>
+        <v>70273</v>
       </c>
       <c r="D11" s="3">
-        <v>35170</v>
+        <v>285400</v>
       </c>
       <c r="E11">
         <v>18000</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
         <v>1</v>
       </c>
       <c r="G11">
@@ -3983,23 +4006,23 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="12.75">
+    <row r="12" spans="1:8" ht="13.5" thickBot="1">
       <c r="A12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="3">
-        <v>5300000</v>
+        <v>594</v>
+      </c>
+      <c r="B12" s="101">
+        <v>974666</v>
       </c>
       <c r="C12" s="3">
-        <v>70273</v>
+        <v>9251</v>
       </c>
       <c r="D12" s="3">
-        <v>285400</v>
+        <v>35170</v>
       </c>
       <c r="E12">
         <v>18000</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
@@ -4009,12 +4032,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="12.75">
+    <row r="13" spans="1:8" ht="13.5" thickBot="1">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="3">
-        <v>10300000</v>
+      <c r="B13" s="102">
+        <v>10694681</v>
       </c>
       <c r="C13" s="3">
         <v>92090</v>
@@ -4035,12 +4058,12 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="12.75">
+    <row r="14" spans="1:8" ht="13.5" thickBot="1">
       <c r="A14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="3">
-        <v>37700000</v>
+      <c r="B14" s="101">
+        <v>36559233</v>
       </c>
       <c r="C14" s="3">
         <v>312685</v>
@@ -4061,12 +4084,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="12.75">
+    <row r="15" spans="1:8" ht="13.5" thickBot="1">
       <c r="A15" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="B15" s="3">
-        <v>3900000</v>
+      <c r="B15" s="102">
+        <v>3868159</v>
       </c>
       <c r="C15" s="3">
         <v>56594</v>
@@ -4081,11 +4104,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="12.75">
+    <row r="16" spans="1:8" ht="13.5" thickBot="1">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="102">
         <v>1000000</v>
       </c>
       <c r="C16" s="4">
@@ -4107,12 +4130,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="12.75">
+    <row r="17" spans="1:8" ht="13.5" thickBot="1">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="3">
-        <v>11700000</v>
+      <c r="B17" s="101">
+        <v>11850296</v>
       </c>
       <c r="C17" s="4">
         <v>30528</v>
@@ -4133,12 +4156,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="12.75">
+    <row r="18" spans="1:8" ht="13.5" thickBot="1">
       <c r="A18" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="B18" s="3">
-        <v>5500000</v>
+      <c r="B18" s="102">
+        <v>5572272</v>
       </c>
       <c r="C18" s="3">
         <v>323802</v>
@@ -4156,91 +4179,94 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="12.75">
+    <row r="19" spans="1:8" ht="13.5" thickBot="1">
       <c r="A19" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="3">
-        <v>2800000</v>
+        <v>37</v>
+      </c>
+      <c r="B19" s="102">
+        <v>85518661</v>
       </c>
       <c r="C19" s="3">
-        <v>28748</v>
+        <v>783562</v>
       </c>
       <c r="D19" s="3">
-        <v>11710</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="12.75">
+        <v>756600</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="13.5" thickBot="1">
       <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="102">
+        <v>10905028</v>
+      </c>
+      <c r="C20" s="3">
+        <v>78867</v>
+      </c>
+      <c r="D20" s="3">
+        <v>151270</v>
+      </c>
+      <c r="F20" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="13.5" thickBot="1">
+      <c r="A21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="3">
-        <v>6700000</v>
-      </c>
-      <c r="C20" s="3">
+      <c r="B21" s="101">
+        <v>6441421</v>
+      </c>
+      <c r="C21" s="3">
         <v>110994</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D21" s="3">
         <v>103390</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F21" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="12.75">
-      <c r="A21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3">
-        <v>10900000</v>
-      </c>
-      <c r="C21" s="3">
-        <v>78867</v>
-      </c>
-      <c r="D21" s="3">
-        <v>151270</v>
-      </c>
-      <c r="F21" s="2">
+    <row r="22" spans="1:8" ht="13.5" thickBot="1">
+      <c r="A22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="102">
+        <v>2888278</v>
+      </c>
+      <c r="C22" s="3">
+        <v>65300</v>
+      </c>
+      <c r="D22" s="3">
+        <v>101610</v>
+      </c>
+      <c r="F22" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="12.75">
-      <c r="A22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="3">
-        <v>5400000</v>
-      </c>
-      <c r="C22" s="3">
-        <v>49035</v>
-      </c>
-      <c r="D22" s="3">
-        <v>43290</v>
-      </c>
-      <c r="F22" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="12.75">
+    <row r="23" spans="1:8" ht="13.5" thickBot="1">
       <c r="A23" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="3">
-        <v>1300000</v>
+        <v>25</v>
+      </c>
+      <c r="B23" s="101">
+        <v>19055364</v>
       </c>
       <c r="C23" s="3">
-        <v>45339</v>
+        <v>238391</v>
       </c>
       <c r="D23" s="3">
-        <v>46180</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="12.75">
+        <v>97360</v>
+      </c>
+      <c r="F23" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="13.5" thickBot="1">
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="3">
-        <v>9600000</v>
+      <c r="B24" s="102">
+        <v>9562065</v>
       </c>
       <c r="C24" s="3">
         <v>93030</v>
@@ -4249,126 +4275,123 @@
         <v>94080</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="12.75">
+    <row r="25" spans="1:8" ht="13.5" thickBot="1">
       <c r="A25" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="3">
-        <v>1800000</v>
+        <v>27</v>
+      </c>
+      <c r="B25" s="102">
+        <v>10569709</v>
       </c>
       <c r="C25" s="3">
-        <v>64589</v>
+        <v>450295</v>
       </c>
       <c r="D25" s="3">
-        <v>51910</v>
+        <v>83480</v>
       </c>
       <c r="F25" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="12.75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="13.5" thickBot="1">
       <c r="A26" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="3">
-        <v>2800000</v>
+        <v>29</v>
+      </c>
+      <c r="B26" s="102">
+        <v>6586476</v>
       </c>
       <c r="C26" s="3">
-        <v>65300</v>
+        <v>77474</v>
       </c>
       <c r="D26" s="3">
-        <v>101610</v>
+        <v>53370</v>
       </c>
       <c r="F26" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="12.75">
+    <row r="27" spans="1:8" ht="13.5" thickBot="1">
       <c r="A27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="3">
-        <v>19000000</v>
+        <v>30</v>
+      </c>
+      <c r="B27" s="102">
+        <v>1869570</v>
       </c>
       <c r="C27" s="3">
-        <v>238391</v>
+        <v>64589</v>
       </c>
       <c r="D27" s="3">
-        <v>97360</v>
+        <v>51910</v>
       </c>
       <c r="F27" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="12.75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="13.5" thickBot="1">
       <c r="A28" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="3">
-        <v>6700000</v>
+        <v>31</v>
+      </c>
+      <c r="B28" s="102">
+        <v>1372341</v>
       </c>
       <c r="C28" s="3">
-        <v>77474</v>
+        <v>45339</v>
       </c>
       <c r="D28" s="3">
-        <v>53370</v>
-      </c>
-      <c r="F28" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="12.75">
+        <v>46180</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="13.5" thickBot="1">
       <c r="A29" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="101">
+        <v>5422069</v>
+      </c>
+      <c r="C29" s="3">
+        <v>49035</v>
+      </c>
+      <c r="D29" s="3">
+        <v>43290</v>
+      </c>
+      <c r="F29" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="13.5" thickBot="1">
+      <c r="A30" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B29" s="3">
-        <v>2100000</v>
-      </c>
-      <c r="C29" s="3">
+      <c r="B30" s="102">
+        <v>2127400</v>
+      </c>
+      <c r="C30" s="3">
         <v>20273</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D30" s="3">
         <v>15560</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F30" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="12.75">
-      <c r="A30" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="3">
-        <v>10600000</v>
-      </c>
-      <c r="C30" s="3">
-        <v>450295</v>
-      </c>
-      <c r="D30" s="3">
-        <v>83480</v>
-      </c>
-      <c r="F30" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="12.75">
+    <row r="31" spans="1:8" ht="13.5" thickBot="1">
       <c r="A31" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" s="3">
-        <v>86500000</v>
+        <v>36</v>
+      </c>
+      <c r="B31" s="101">
+        <v>2377128</v>
       </c>
       <c r="C31" s="3">
-        <v>783562</v>
+        <v>28748</v>
       </c>
       <c r="D31" s="3">
-        <v>756600</v>
+        <v>11710</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H31" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
-      <sortCondition descending="1" ref="E1:E31"/>
+      <sortCondition descending="1" ref="E2:E31"/>
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
@@ -14741,7 +14764,7 @@
       <c r="A2" s="37" t="s">
         <v>365</v>
       </c>
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="95" t="s">
         <v>366</v>
       </c>
       <c r="C2" s="94"/>
@@ -14768,7 +14791,7 @@
       <c r="A3" s="37" t="s">
         <v>367</v>
       </c>
-      <c r="B3" s="98">
+      <c r="B3" s="96">
         <v>45586.958333333336</v>
       </c>
       <c r="C3" s="94"/>
@@ -14844,7 +14867,7 @@
       <c r="U5" s="17"/>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="97" t="s">
+      <c r="A6" s="95" t="s">
         <v>371</v>
       </c>
       <c r="B6" s="94"/>
@@ -14924,46 +14947,46 @@
       <c r="A9" s="40" t="s">
         <v>375</v>
       </c>
-      <c r="B9" s="95">
+      <c r="B9" s="97">
         <v>2011</v>
       </c>
-      <c r="C9" s="96"/>
-      <c r="D9" s="95">
+      <c r="C9" s="98"/>
+      <c r="D9" s="97">
         <v>2012</v>
       </c>
-      <c r="E9" s="96"/>
-      <c r="F9" s="95">
+      <c r="E9" s="98"/>
+      <c r="F9" s="97">
         <v>2013</v>
       </c>
-      <c r="G9" s="96"/>
-      <c r="H9" s="95">
+      <c r="G9" s="98"/>
+      <c r="H9" s="97">
         <v>2014</v>
       </c>
-      <c r="I9" s="96"/>
-      <c r="J9" s="95">
+      <c r="I9" s="98"/>
+      <c r="J9" s="97">
         <v>2015</v>
       </c>
-      <c r="K9" s="96"/>
-      <c r="L9" s="95">
+      <c r="K9" s="98"/>
+      <c r="L9" s="97">
         <v>2016</v>
       </c>
-      <c r="M9" s="96"/>
-      <c r="N9" s="95">
+      <c r="M9" s="98"/>
+      <c r="N9" s="97">
         <v>2017</v>
       </c>
-      <c r="O9" s="96"/>
-      <c r="P9" s="95">
+      <c r="O9" s="98"/>
+      <c r="P9" s="97">
         <v>2018</v>
       </c>
-      <c r="Q9" s="96"/>
-      <c r="R9" s="95">
+      <c r="Q9" s="98"/>
+      <c r="R9" s="97">
         <v>2019</v>
       </c>
-      <c r="S9" s="96"/>
-      <c r="T9" s="95">
+      <c r="S9" s="98"/>
+      <c r="T9" s="97">
         <v>2020</v>
       </c>
-      <c r="U9" s="96"/>
+      <c r="U9" s="98"/>
     </row>
     <row r="10" spans="1:21">
       <c r="A10" s="41" t="s">
@@ -16831,12 +16854,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="P9:Q9"/>
     <mergeCell ref="R9:S9"/>
@@ -16848,6 +16865,12 @@
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="N9:O9"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>

</xml_diff>